<commit_message>
setup for linux ros 2
</commit_message>
<xml_diff>
--- a/Greyform-linux/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
+++ b/Greyform-linux/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="103">
   <si>
     <t>Marking type</t>
   </si>
@@ -24,6 +24,300 @@
     <t>Point number/name</t>
   </si>
   <si>
+    <t>Position X (m)</t>
+  </si>
+  <si>
+    <t>Position Y (m)</t>
+  </si>
+  <si>
+    <t>Position Z (m)</t>
+  </si>
+  <si>
+    <t>Wall Number</t>
+  </si>
+  <si>
+    <t>Shape type</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Quadrant</t>
+  </si>
+  <si>
+    <t>Unnamed : 9</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>Orientation</t>
+  </si>
+  <si>
+    <t>Diameter</t>
+  </si>
+  <si>
+    <t>Tile</t>
+  </si>
+  <si>
+    <t>TMP1S2e4:TMP1S2e4:1155212</t>
+  </si>
+  <si>
+    <t>TMP1S2f1:TMP1S2f1:1155220</t>
+  </si>
+  <si>
+    <t>TMP1S2f2:TMP1S2f2:1155219</t>
+  </si>
+  <si>
+    <t>TMP1S2f3:TMP1S2f3:1155218</t>
+  </si>
+  <si>
+    <t>TMP1S2f4:TMP1S2f4:1155217</t>
+  </si>
+  <si>
+    <t>TMP1S2e1:TMP1S2e1:1155215</t>
+  </si>
+  <si>
+    <t>TMP1S2e2:TMP1S2e2:1155214</t>
+  </si>
+  <si>
+    <t>TMP1S2e3:TMP1S2e3:1155213</t>
+  </si>
+  <si>
+    <t>TMP1S2d1:TMP1S2d1:1155210</t>
+  </si>
+  <si>
+    <t>TMP1S2d2:TMP1S2d2:1155209</t>
+  </si>
+  <si>
+    <t>TMP1S2d3:TMP1S2d3:1155208</t>
+  </si>
+  <si>
+    <t>TMP1S2d4:TMP1S2d4:1155207</t>
+  </si>
+  <si>
+    <t>TMP1S2c1:TMP1S2c1:1155205</t>
+  </si>
+  <si>
+    <t>TMP1S2c2:TMP1S2c2:1155204</t>
+  </si>
+  <si>
+    <t>TMP1S2c4:TMP1S2c4:1155202</t>
+  </si>
+  <si>
+    <t>TMP1S2c3:TMP1S2c3:1155203</t>
+  </si>
+  <si>
+    <t>TMP1S2b2:TMP1S2b2:1155199</t>
+  </si>
+  <si>
+    <t>TMP1S2b3:TMP1S2b3:1155198</t>
+  </si>
+  <si>
+    <t>TMP1S2b4:TMP1S2b4:1155197</t>
+  </si>
+  <si>
+    <t>TMP1S2a1:TMP1S2a1:1155195</t>
+  </si>
+  <si>
+    <t>TMP1S2a2:TMP1S2a2:1155194</t>
+  </si>
+  <si>
+    <t>TMP1S2a3:TMP1S2a3:1155193</t>
+  </si>
+  <si>
+    <t>TMP1S2a4:TMP1S2a4:1155192</t>
+  </si>
+  <si>
+    <t>TMP1S2b1:TMP1S2b1:1155200</t>
+  </si>
+  <si>
+    <t>TMP2S2b2:TMP2S2b2:1155222</t>
+  </si>
+  <si>
+    <t>TMP2S2a2:TMP2S2a2:1155224</t>
+  </si>
+  <si>
+    <t>TMP2S2b1:TMP2S2b1:1155223</t>
+  </si>
+  <si>
+    <t>TMP2S2a1:TMP2S2a1:1155225</t>
+  </si>
+  <si>
+    <t>TMP3S2b3:TMP3S2b3:1155228</t>
+  </si>
+  <si>
+    <t>TMP3S2b1:TMP3S2b1:1155229</t>
+  </si>
+  <si>
+    <t>TMP3S2a4:TMP3S2a4:1155231</t>
+  </si>
+  <si>
+    <t>TMP3S2a3:TMP3S2a3:1155232</t>
+  </si>
+  <si>
+    <t>TMP3S2a2:TMP3S2a2:1155233</t>
+  </si>
+  <si>
+    <t>TMP3S2a1:TMP3S2a1:1155234</t>
+  </si>
+  <si>
+    <t>TMP3S2b4:TMP3S2b4:1155227</t>
+  </si>
+  <si>
+    <t>TMP3S2b2:TMP3S2b2:1155230</t>
+  </si>
+  <si>
+    <t>TMP4S2a4:TMP4S2a4:1155237</t>
+  </si>
+  <si>
+    <t>TMP4S2a1:TMP4S2a1:1155243</t>
+  </si>
+  <si>
+    <t>TMP4S2a2:TMP4S2a2:1155242</t>
+  </si>
+  <si>
+    <t>TMP4S2a3:TMP4S2a3:1155241</t>
+  </si>
+  <si>
+    <t>TMP5S2b3:TMP5S2b3:1155248</t>
+  </si>
+  <si>
+    <t>TMP5S2a2:TMP5S2a2:1155249</t>
+  </si>
+  <si>
+    <t>TMP5S2a3:TMP5S2a3:1155247</t>
+  </si>
+  <si>
+    <t>TMP5S2b2:TMP5S2b2:1155250</t>
+  </si>
+  <si>
+    <t>TMP5S2b1:TMP5S2b1:1155251</t>
+  </si>
+  <si>
+    <t>TMP5S2a1:TMP5S2a1:1155252</t>
+  </si>
+  <si>
+    <t>TMP5S2b4:TMP5S2b4:1155246</t>
+  </si>
+  <si>
+    <t>TMP5S2a4:TMP5S2a4:1155245</t>
+  </si>
+  <si>
+    <t>TMP4S2b2:TMP4S2b2:1155239</t>
+  </si>
+  <si>
+    <t>TMP4S2b3:TMP4S2b3:1155238</t>
+  </si>
+  <si>
+    <t>TMP4S2b4:TMP4S2b4:1155236</t>
+  </si>
+  <si>
+    <t>TMP4S2b1:TMP4S2b1:1155240</t>
+  </si>
+  <si>
+    <t>TMP6S2b1:TMP6S2b1:1155262</t>
+  </si>
+  <si>
+    <t>TMP6S2b2:TMP6S2b2:1155261</t>
+  </si>
+  <si>
+    <t>TMP6S2b4:TMP6S2b4:1155259</t>
+  </si>
+  <si>
+    <t>TMP6S2b3:TMP6S2b3:1155260</t>
+  </si>
+  <si>
+    <t>TMP6S2a2:TMP6S2a2:1155256</t>
+  </si>
+  <si>
+    <t>TMP6S2a4:TMP6S2a4:1155255</t>
+  </si>
+  <si>
+    <t>TMP6S2a3:TMP6S2a3:1155254</t>
+  </si>
+  <si>
+    <t>TMP6S2a1:TMP6S2a1:1155257</t>
+  </si>
+  <si>
+    <t>TMP7S2c2:TMP7S2c2:1155275</t>
+  </si>
+  <si>
+    <t>TMP7S2b3:TMP7S2b3:1155264</t>
+  </si>
+  <si>
+    <t>TMP7S2b2:TMP7S2b2:1155265</t>
+  </si>
+  <si>
+    <t>TMP7S2b1:TMP7S2b1:1155266</t>
+  </si>
+  <si>
+    <t>TMP7S2a3:TMP7S2a3:1155267</t>
+  </si>
+  <si>
+    <t>TMP7S2a2:TMP7S2a2:1155268</t>
+  </si>
+  <si>
+    <t>TMP7S2a1:TMP7S2a1:1155269</t>
+  </si>
+  <si>
+    <t>TMP7S2d1:TMP7S2d1:1155271</t>
+  </si>
+  <si>
+    <t>TMP7S2d2:TMP7S2d2:1155272</t>
+  </si>
+  <si>
+    <t>TMP7S2d3:TMP7S2d3:1155273</t>
+  </si>
+  <si>
+    <t>TMP7S2c3:TMP7S2c3:1155274</t>
+  </si>
+  <si>
+    <t>TMP7S2c1:TMP7S2c1:1155276</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>blank</t>
+  </si>
+  <si>
+    <t>Fitting</t>
+  </si>
+  <si>
+    <t>BSS.HAND SHOWER SET.MASTER BATH:BSS.HAND SHOWER SET.MASTER BATH:1091130</t>
+  </si>
+  <si>
+    <t>BSS.GESSI.SM.49079:29046000:1090989</t>
+  </si>
+  <si>
+    <t>BSS.Bottle Trap:BSS.Bottle trap:1018126</t>
+  </si>
+  <si>
+    <t>BSS.LAUFEN.WC.820714:820959000 White:1091064</t>
+  </si>
+  <si>
+    <t>BSS.TECE.AP.9240402:Flush Plate:1091024</t>
+  </si>
+  <si>
+    <t>BSS.GESSI,BM.49001:Default:1090988</t>
+  </si>
+  <si>
+    <t>BSS.MONIC.BIB TAP.T-4L:BIB TAP:1090961</t>
+  </si>
+  <si>
+    <t>BSS.MIRROR CABINET.C5-MASTER BATH:BSS.MIRROR CABINET.C5-MASTER BATH:1090945</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>Position X (mm)</t>
   </si>
   <si>
@@ -31,297 +325,6 @@
   </si>
   <si>
     <t>Position Z (mm)</t>
-  </si>
-  <si>
-    <t>Wall Number</t>
-  </si>
-  <si>
-    <t>Shape type</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Quadrant</t>
-  </si>
-  <si>
-    <t>Unnamed : 9</t>
-  </si>
-  <si>
-    <t>Width</t>
-  </si>
-  <si>
-    <t>Height</t>
-  </si>
-  <si>
-    <t>Orientation</t>
-  </si>
-  <si>
-    <t>Diameter</t>
-  </si>
-  <si>
-    <t>Tile</t>
-  </si>
-  <si>
-    <t>TMP1S2c3:TMP1S2c3:1155203</t>
-  </si>
-  <si>
-    <t>TMP1S2d1:TMP1S2d1:1155210</t>
-  </si>
-  <si>
-    <t>TMP1S2d2:TMP1S2d2:1155209</t>
-  </si>
-  <si>
-    <t>TMP1S2d3:TMP1S2d3:1155208</t>
-  </si>
-  <si>
-    <t>TMP1S2d4:TMP1S2d4:1155207</t>
-  </si>
-  <si>
-    <t>TMP1S2c1:TMP1S2c1:1155205</t>
-  </si>
-  <si>
-    <t>TMP1S2c2:TMP1S2c2:1155204</t>
-  </si>
-  <si>
-    <t>TMP1S2e2:TMP1S2e2:1155214</t>
-  </si>
-  <si>
-    <t>TMP1S2c4:TMP1S2c4:1155202</t>
-  </si>
-  <si>
-    <t>TMP1S2b1:TMP1S2b1:1155200</t>
-  </si>
-  <si>
-    <t>TMP1S2b2:TMP1S2b2:1155199</t>
-  </si>
-  <si>
-    <t>TMP1S2b3:TMP1S2b3:1155198</t>
-  </si>
-  <si>
-    <t>TMP1S2b4:TMP1S2b4:1155197</t>
-  </si>
-  <si>
-    <t>TMP1S2a1:TMP1S2a1:1155195</t>
-  </si>
-  <si>
-    <t>TMP1S2a2:TMP1S2a2:1155194</t>
-  </si>
-  <si>
-    <t>TMP1S2a3:TMP1S2a3:1155193</t>
-  </si>
-  <si>
-    <t>TMP1S2a4:TMP1S2a4:1155192</t>
-  </si>
-  <si>
-    <t>TMP1S2e1:TMP1S2e1:1155215</t>
-  </si>
-  <si>
-    <t>TMP1S2f4:TMP1S2f4:1155217</t>
-  </si>
-  <si>
-    <t>TMP1S2f3:TMP1S2f3:1155218</t>
-  </si>
-  <si>
-    <t>TMP1S2f2:TMP1S2f2:1155219</t>
-  </si>
-  <si>
-    <t>TMP1S2f1:TMP1S2f1:1155220</t>
-  </si>
-  <si>
-    <t>TMP1S2e4:TMP1S2e4:1155212</t>
-  </si>
-  <si>
-    <t>TMP1S2e3:TMP1S2e3:1155213</t>
-  </si>
-  <si>
-    <t>TMP2S2b2:TMP2S2b2:1155222</t>
-  </si>
-  <si>
-    <t>TMP2S2b1:TMP2S2b1:1155223</t>
-  </si>
-  <si>
-    <t>TMP2S2c1:TMP2S2c1:1156963</t>
-  </si>
-  <si>
-    <t>TMP2S2c2:TMP2S2c2:1156962</t>
-  </si>
-  <si>
-    <t>TMP2S2a2:TMP2S2a2:1155224</t>
-  </si>
-  <si>
-    <t>TMP2S2a1:TMP2S2a1:1155225</t>
-  </si>
-  <si>
-    <t>TMP3S2b3:TMP3S2b3:1155228</t>
-  </si>
-  <si>
-    <t>TMP3S2b1:TMP3S2b1:1155229</t>
-  </si>
-  <si>
-    <t>TMP3S2b2:TMP3S2b2:1155230</t>
-  </si>
-  <si>
-    <t>TMP3S2a3:TMP3S2a3:1155232</t>
-  </si>
-  <si>
-    <t>TMP3S2a2:TMP3S2a2:1155233</t>
-  </si>
-  <si>
-    <t>TMP3S2a1:TMP3S2a1:1155234</t>
-  </si>
-  <si>
-    <t>TMP3S2a4:TMP3S2a4:1155231</t>
-  </si>
-  <si>
-    <t>TMP3S2b4:TMP3S2b4:1155227</t>
-  </si>
-  <si>
-    <t>TMP4S2a4:TMP4S2a4:1155237</t>
-  </si>
-  <si>
-    <t>TMP4S2a1:TMP4S2a1:1155243</t>
-  </si>
-  <si>
-    <t>TMP4S2a3:TMP4S2a3:1155241</t>
-  </si>
-  <si>
-    <t>TMP4S2a2:TMP4S2a2:1155242</t>
-  </si>
-  <si>
-    <t>TMP5S2b1:TMP5S2b1:1155251</t>
-  </si>
-  <si>
-    <t>TMP5S2b2:TMP5S2b2:1155250</t>
-  </si>
-  <si>
-    <t>TMP5S2a2:TMP5S2a2:1155249</t>
-  </si>
-  <si>
-    <t>TMP5S2b3:TMP5S2b3:1155248</t>
-  </si>
-  <si>
-    <t>TMP5S2a3:TMP5S2a3:1155247</t>
-  </si>
-  <si>
-    <t>TMP5S2b4:TMP5S2b4:1155246</t>
-  </si>
-  <si>
-    <t>TMP5S2a4:TMP5S2a4:1155245</t>
-  </si>
-  <si>
-    <t>TMP5S2a1:TMP5S2a1:1155252</t>
-  </si>
-  <si>
-    <t>TMP4S2b2:TMP4S2b2:1155239</t>
-  </si>
-  <si>
-    <t>TMP4S2b1:TMP4S2b1:1155240</t>
-  </si>
-  <si>
-    <t>TMP4S2b4:TMP4S2b4:1155236</t>
-  </si>
-  <si>
-    <t>TMP4S2b3:TMP4S2b3:1155238</t>
-  </si>
-  <si>
-    <t>TMP6S2b1:TMP6S2b1:1155262</t>
-  </si>
-  <si>
-    <t>TMP6S2b3:TMP6S2b3:1155260</t>
-  </si>
-  <si>
-    <t>TMP6S2b2:TMP6S2b2:1155261</t>
-  </si>
-  <si>
-    <t>TMP6S2a1:TMP6S2a1:1155257</t>
-  </si>
-  <si>
-    <t>TMP6S2a2:TMP6S2a2:1155256</t>
-  </si>
-  <si>
-    <t>TMP6S2a4:TMP6S2a4:1155255</t>
-  </si>
-  <si>
-    <t>TMP6S2a3:TMP6S2a3:1155254</t>
-  </si>
-  <si>
-    <t>TMP6S2b4:TMP6S2b4:1155259</t>
-  </si>
-  <si>
-    <t>TMP7S2c1:TMP7S2c1:1155276</t>
-  </si>
-  <si>
-    <t>TMP7S2c2:TMP7S2c2:1155275</t>
-  </si>
-  <si>
-    <t>TMP7S2c3:TMP7S2c3:1155274</t>
-  </si>
-  <si>
-    <t>TMP7S2d3:TMP7S2d3:1155273</t>
-  </si>
-  <si>
-    <t>TMP7S2d2:TMP7S2d2:1155272</t>
-  </si>
-  <si>
-    <t>TMP7S2a1:TMP7S2a1:1155269</t>
-  </si>
-  <si>
-    <t>TMP7S2a2:TMP7S2a2:1155268</t>
-  </si>
-  <si>
-    <t>TMP7S2a3:TMP7S2a3:1155267</t>
-  </si>
-  <si>
-    <t>TMP7S2b1:TMP7S2b1:1155266</t>
-  </si>
-  <si>
-    <t>TMP7S2b3:TMP7S2b3:1155264</t>
-  </si>
-  <si>
-    <t>TMP7S2d1:TMP7S2d1:1155271</t>
-  </si>
-  <si>
-    <t>TMP7S2b2:TMP7S2b2:1155265</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>+</t>
-  </si>
-  <si>
-    <t>blank</t>
-  </si>
-  <si>
-    <t>Fitting</t>
-  </si>
-  <si>
-    <t>BSS.HAND SHOWER SET.MASTER BATH:BSS.HAND SHOWER SET.MASTER BATH:1091130</t>
-  </si>
-  <si>
-    <t>BSS.GESSI.SM.49079:29046000:1090989</t>
-  </si>
-  <si>
-    <t>BSS.LAUFEN.WC.820714:820959000 White:1091064</t>
-  </si>
-  <si>
-    <t>BSS.TECE.AP.9240402:Flush Plate:1091024</t>
-  </si>
-  <si>
-    <t>BSS.GESSI,BM.49001:Default:1090988</t>
-  </si>
-  <si>
-    <t>BSS.Bottle Trap:BSS.Bottle trap:1018126</t>
-  </si>
-  <si>
-    <t>BSS.MIRROR CABINET.C5-MASTER BATH:BSS.MIRROR CABINET.C5-MASTER BATH:1090945</t>
-  </si>
-  <si>
-    <t>BSS.MONIC.BIB TAP.T-4L:BIB TAP:1090961</t>
-  </si>
-  <si>
-    <t>6</t>
   </si>
 </sst>
 </file>
@@ -679,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -728,7 +731,7 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="1">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -740,10 +743,10 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>-30</v>
+        <v>0.49</v>
       </c>
       <c r="F2">
-        <v>-175</v>
+        <v>1.025</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -752,21 +755,21 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="L2">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M2">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="1">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -778,10 +781,10 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>470</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F3">
-        <v>1025</v>
+        <v>1.025</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -790,21 +793,21 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M3">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -816,10 +819,10 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>470</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F4">
-        <v>425</v>
+        <v>0.425</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -828,21 +831,21 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M4">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="1">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -854,10 +857,10 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>470</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F5">
-        <v>-175</v>
+        <v>-0.175</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -866,21 +869,21 @@
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J5">
         <v>1</v>
       </c>
       <c r="L5">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M5">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="1">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -892,10 +895,10 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>470</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F6">
-        <v>-775</v>
+        <v>-0.775</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -904,21 +907,21 @@
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J6">
         <v>1</v>
       </c>
       <c r="L6">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M6">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="1">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -930,10 +933,10 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>-30</v>
+        <v>0.49</v>
       </c>
       <c r="F7">
-        <v>1025</v>
+        <v>1.025</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -942,21 +945,21 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="L7">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M7">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="1">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
@@ -968,10 +971,10 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>-30</v>
+        <v>0.49</v>
       </c>
       <c r="F8">
-        <v>425</v>
+        <v>0.425</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -980,21 +983,21 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J8">
         <v>1</v>
       </c>
       <c r="L8">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M8">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="1">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
@@ -1006,10 +1009,10 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>490</v>
+        <v>0.49</v>
       </c>
       <c r="F9">
-        <v>425</v>
+        <v>-0.175</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -1018,21 +1021,21 @@
         <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J9">
         <v>1</v>
       </c>
       <c r="L9">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M9">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="1">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
@@ -1044,10 +1047,10 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>-30</v>
+        <v>0.47</v>
       </c>
       <c r="F10">
-        <v>-775</v>
+        <v>1.025</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -1056,21 +1059,21 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J10">
         <v>1</v>
       </c>
       <c r="L10">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M10">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="1">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B11" t="s">
         <v>14</v>
@@ -1082,10 +1085,10 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>-350</v>
+        <v>0.47</v>
       </c>
       <c r="F11">
-        <v>1025</v>
+        <v>0.425</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -1094,21 +1097,21 @@
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M11">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="1">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -1120,10 +1123,10 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>-350</v>
+        <v>0.47</v>
       </c>
       <c r="F12">
-        <v>425</v>
+        <v>-0.175</v>
       </c>
       <c r="G12">
         <v>1</v>
@@ -1132,21 +1135,21 @@
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J12">
         <v>1</v>
       </c>
       <c r="L12">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M12">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="1">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1158,10 +1161,10 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>-350</v>
+        <v>0.47</v>
       </c>
       <c r="F13">
-        <v>-175</v>
+        <v>-0.775</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1170,21 +1173,21 @@
         <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J13">
         <v>1</v>
       </c>
       <c r="L13">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M13">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="1">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
@@ -1196,10 +1199,10 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>-350</v>
+        <v>-0.03</v>
       </c>
       <c r="F14">
-        <v>-775</v>
+        <v>1.025</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1208,21 +1211,21 @@
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J14">
         <v>1</v>
       </c>
       <c r="L14">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M14">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="1">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
@@ -1234,10 +1237,10 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>-1350</v>
+        <v>-0.03</v>
       </c>
       <c r="F15">
-        <v>1025</v>
+        <v>0.425</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1246,21 +1249,21 @@
         <v>1</v>
       </c>
       <c r="I15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J15">
         <v>1</v>
       </c>
       <c r="L15">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M15">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="1">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
@@ -1272,10 +1275,10 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-1350</v>
+        <v>-0.03</v>
       </c>
       <c r="F16">
-        <v>425</v>
+        <v>-0.775</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1284,21 +1287,21 @@
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J16">
         <v>1</v>
       </c>
       <c r="L16">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M16">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="1">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1310,10 +1313,10 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>-1350</v>
+        <v>-0.03</v>
       </c>
       <c r="F17">
-        <v>-175</v>
+        <v>-0.175</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1322,21 +1325,21 @@
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J17">
         <v>1</v>
       </c>
       <c r="L17">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M17">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="1">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -1348,10 +1351,10 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>-1350</v>
+        <v>-0.35</v>
       </c>
       <c r="F18">
-        <v>-775</v>
+        <v>0.425</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1360,21 +1363,21 @@
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J18">
         <v>1</v>
       </c>
       <c r="L18">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M18">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="1">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1386,10 +1389,10 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>490</v>
+        <v>-0.35</v>
       </c>
       <c r="F19">
-        <v>1025</v>
+        <v>-0.175</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1398,21 +1401,21 @@
         <v>1</v>
       </c>
       <c r="I19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J19">
         <v>1</v>
       </c>
       <c r="L19">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M19">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="1">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1424,10 +1427,10 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>935</v>
+        <v>-0.35</v>
       </c>
       <c r="F20">
-        <v>-775</v>
+        <v>-0.775</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1436,21 +1439,21 @@
         <v>1</v>
       </c>
       <c r="I20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J20">
         <v>1</v>
       </c>
       <c r="L20">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M20">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="1">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1462,10 +1465,10 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>935</v>
+        <v>-1.35</v>
       </c>
       <c r="F21">
-        <v>-175</v>
+        <v>1.025</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1474,21 +1477,21 @@
         <v>1</v>
       </c>
       <c r="I21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J21">
         <v>1</v>
       </c>
       <c r="L21">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M21">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="1">
-        <v>187</v>
+        <v>167</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1500,10 +1503,10 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>935</v>
+        <v>-1.35</v>
       </c>
       <c r="F22">
-        <v>425</v>
+        <v>0.425</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1512,21 +1515,21 @@
         <v>1</v>
       </c>
       <c r="I22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J22">
         <v>1</v>
       </c>
       <c r="L22">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M22">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="1">
-        <v>188</v>
+        <v>166</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1538,10 +1541,10 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>935</v>
+        <v>-1.35</v>
       </c>
       <c r="F23">
-        <v>1025</v>
+        <v>-0.175</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -1550,21 +1553,21 @@
         <v>1</v>
       </c>
       <c r="I23" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J23">
         <v>1</v>
       </c>
       <c r="L23">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M23">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="1">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1576,10 +1579,10 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>490</v>
+        <v>-1.35</v>
       </c>
       <c r="F24">
-        <v>1025</v>
+        <v>-0.775</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1588,21 +1591,21 @@
         <v>1</v>
       </c>
       <c r="I24" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J24">
         <v>1</v>
       </c>
       <c r="L24">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M24">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="1">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1614,10 +1617,10 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>490</v>
+        <v>-0.35</v>
       </c>
       <c r="F25">
-        <v>-175</v>
+        <v>1.025</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -1626,16 +1629,16 @@
         <v>1</v>
       </c>
       <c r="I25" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J25">
         <v>1</v>
       </c>
       <c r="L25">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M25">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -1649,13 +1652,13 @@
         <v>39</v>
       </c>
       <c r="D26">
-        <v>-2760</v>
+        <v>-2.76</v>
       </c>
       <c r="E26">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F26">
-        <v>-775</v>
+        <v>-0.775</v>
       </c>
       <c r="G26">
         <v>2</v>
@@ -1664,21 +1667,21 @@
         <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J26">
         <v>1</v>
       </c>
       <c r="L26">
-        <v>1340</v>
+        <v>1.34</v>
       </c>
       <c r="M26">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="27" spans="1:13">
       <c r="A27" s="1">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1687,13 +1690,13 @@
         <v>40</v>
       </c>
       <c r="D27">
-        <v>-2760</v>
+        <v>-2.76</v>
       </c>
       <c r="E27">
-        <v>100</v>
+        <v>-0.5</v>
       </c>
       <c r="F27">
-        <v>-175</v>
+        <v>-0.775</v>
       </c>
       <c r="G27">
         <v>2</v>
@@ -1702,21 +1705,21 @@
         <v>1</v>
       </c>
       <c r="I27" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J27">
         <v>1</v>
       </c>
       <c r="L27">
-        <v>1340</v>
+        <v>1.34</v>
       </c>
       <c r="M27">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="28" spans="1:13">
       <c r="A28" s="1">
-        <v>238</v>
+        <v>190</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1725,13 +1728,13 @@
         <v>41</v>
       </c>
       <c r="D28">
-        <v>-2760</v>
+        <v>-2.76</v>
       </c>
       <c r="E28">
-        <v>150</v>
+        <v>0.1</v>
       </c>
       <c r="F28">
-        <v>1025</v>
+        <v>-0.175</v>
       </c>
       <c r="G28">
         <v>2</v>
@@ -1740,21 +1743,21 @@
         <v>1</v>
       </c>
       <c r="I28" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J28">
         <v>1</v>
       </c>
       <c r="L28">
-        <v>1340</v>
+        <v>1.34</v>
       </c>
       <c r="M28">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="29" spans="1:13">
       <c r="A29" s="1">
-        <v>237</v>
+        <v>192</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1763,13 +1766,13 @@
         <v>42</v>
       </c>
       <c r="D29">
-        <v>-2760</v>
+        <v>-2.76</v>
       </c>
       <c r="E29">
-        <v>150</v>
+        <v>-0.5</v>
       </c>
       <c r="F29">
-        <v>425</v>
+        <v>-0.175</v>
       </c>
       <c r="G29">
         <v>2</v>
@@ -1778,21 +1781,21 @@
         <v>1</v>
       </c>
       <c r="I29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J29">
         <v>1</v>
       </c>
       <c r="L29">
-        <v>1340</v>
+        <v>1.34</v>
       </c>
       <c r="M29">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="1">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1801,36 +1804,36 @@
         <v>43</v>
       </c>
       <c r="D30">
-        <v>-2760</v>
+        <v>1.2</v>
       </c>
       <c r="E30">
-        <v>-500</v>
+        <v>0.445</v>
       </c>
       <c r="F30">
-        <v>-775</v>
+        <v>-0.175</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30">
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J30">
         <v>1</v>
       </c>
       <c r="L30">
-        <v>1340</v>
+        <v>0.96</v>
       </c>
       <c r="M30">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="31" spans="1:13">
       <c r="A31" s="1">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1839,36 +1842,36 @@
         <v>44</v>
       </c>
       <c r="D31">
-        <v>-2760</v>
+        <v>1.2</v>
       </c>
       <c r="E31">
-        <v>-500</v>
+        <v>0.445</v>
       </c>
       <c r="F31">
-        <v>-175</v>
+        <v>1.025</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J31">
         <v>1</v>
       </c>
       <c r="L31">
-        <v>1340</v>
+        <v>0.96</v>
       </c>
       <c r="M31">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="32" spans="1:13">
       <c r="A32" s="1">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1877,13 +1880,13 @@
         <v>45</v>
       </c>
       <c r="D32">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E32">
-        <v>445</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>-175</v>
+        <v>1.025</v>
       </c>
       <c r="G32">
         <v>3</v>
@@ -1892,21 +1895,21 @@
         <v>1</v>
       </c>
       <c r="I32" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J32">
         <v>1</v>
       </c>
       <c r="L32">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M32">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="1">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1915,13 +1918,13 @@
         <v>46</v>
       </c>
       <c r="D33">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E33">
-        <v>445</v>
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>1025</v>
+        <v>-0.175</v>
       </c>
       <c r="G33">
         <v>3</v>
@@ -1930,21 +1933,21 @@
         <v>1</v>
       </c>
       <c r="I33" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J33">
         <v>1</v>
       </c>
       <c r="L33">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M33">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="1">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1953,13 +1956,13 @@
         <v>47</v>
       </c>
       <c r="D34">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E34">
-        <v>445</v>
+        <v>0</v>
       </c>
       <c r="F34">
-        <v>425</v>
+        <v>0.425</v>
       </c>
       <c r="G34">
         <v>3</v>
@@ -1968,21 +1971,21 @@
         <v>1</v>
       </c>
       <c r="I34" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J34">
         <v>1</v>
       </c>
       <c r="L34">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M34">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="35" spans="1:13">
       <c r="A35" s="1">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -1991,13 +1994,13 @@
         <v>48</v>
       </c>
       <c r="D35">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E35">
         <v>0</v>
       </c>
       <c r="F35">
-        <v>-175</v>
+        <v>1.025</v>
       </c>
       <c r="G35">
         <v>3</v>
@@ -2006,21 +2009,21 @@
         <v>1</v>
       </c>
       <c r="I35" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J35">
         <v>1</v>
       </c>
       <c r="L35">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M35">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="1">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -2029,13 +2032,13 @@
         <v>49</v>
       </c>
       <c r="D36">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>0.445</v>
       </c>
       <c r="F36">
-        <v>425</v>
+        <v>-0.775</v>
       </c>
       <c r="G36">
         <v>3</v>
@@ -2044,21 +2047,21 @@
         <v>1</v>
       </c>
       <c r="I36" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J36">
         <v>1</v>
       </c>
       <c r="L36">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M36">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="37" spans="1:13">
       <c r="A37" s="1">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -2067,13 +2070,13 @@
         <v>50</v>
       </c>
       <c r="D37">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>0.445</v>
       </c>
       <c r="F37">
-        <v>1025</v>
+        <v>0.425</v>
       </c>
       <c r="G37">
         <v>3</v>
@@ -2082,21 +2085,21 @@
         <v>1</v>
       </c>
       <c r="I37" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J37">
         <v>1</v>
       </c>
       <c r="L37">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M37">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="38" spans="1:13">
       <c r="A38" s="1">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -2105,36 +2108,36 @@
         <v>51</v>
       </c>
       <c r="D38">
-        <v>1200</v>
+        <v>0.96</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="F38">
-        <v>1025</v>
+        <v>-0.775</v>
       </c>
       <c r="G38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H38">
         <v>1</v>
       </c>
       <c r="I38" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J38">
         <v>1</v>
       </c>
       <c r="L38">
-        <v>960</v>
+        <v>0.592</v>
       </c>
       <c r="M38">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="39" spans="1:13">
       <c r="A39" s="1">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
@@ -2143,36 +2146,36 @@
         <v>52</v>
       </c>
       <c r="D39">
-        <v>1200</v>
+        <v>0.96</v>
       </c>
       <c r="E39">
-        <v>445</v>
+        <v>-0.3</v>
       </c>
       <c r="F39">
-        <v>-775</v>
+        <v>1.025</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H39">
         <v>1</v>
       </c>
       <c r="I39" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J39">
         <v>1</v>
       </c>
       <c r="L39">
-        <v>960</v>
+        <v>0.592</v>
       </c>
       <c r="M39">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="40" spans="1:13">
       <c r="A40" s="1">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
@@ -2181,13 +2184,13 @@
         <v>53</v>
       </c>
       <c r="D40">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="E40">
-        <v>-300</v>
+        <v>-0.3</v>
       </c>
       <c r="F40">
-        <v>-775</v>
+        <v>0.425</v>
       </c>
       <c r="G40">
         <v>4</v>
@@ -2196,21 +2199,21 @@
         <v>1</v>
       </c>
       <c r="I40" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J40">
         <v>1</v>
       </c>
       <c r="L40">
-        <v>592</v>
+        <v>0.592</v>
       </c>
       <c r="M40">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="41" spans="1:13">
       <c r="A41" s="1">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
@@ -2219,13 +2222,13 @@
         <v>54</v>
       </c>
       <c r="D41">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="E41">
-        <v>-300</v>
+        <v>-0.3</v>
       </c>
       <c r="F41">
-        <v>1025</v>
+        <v>-0.175</v>
       </c>
       <c r="G41">
         <v>4</v>
@@ -2234,21 +2237,21 @@
         <v>1</v>
       </c>
       <c r="I41" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J41">
         <v>1</v>
       </c>
       <c r="L41">
-        <v>592</v>
+        <v>0.592</v>
       </c>
       <c r="M41">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="1">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B42" t="s">
         <v>14</v>
@@ -2257,36 +2260,36 @@
         <v>55</v>
       </c>
       <c r="D42">
-        <v>960</v>
+        <v>0.6</v>
       </c>
       <c r="E42">
-        <v>-300</v>
+        <v>-0.45</v>
       </c>
       <c r="F42">
-        <v>-175</v>
+        <v>-0.025</v>
       </c>
       <c r="G42">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H42">
         <v>1</v>
       </c>
       <c r="I42" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J42">
         <v>1</v>
       </c>
       <c r="L42">
-        <v>592</v>
+        <v>1.94</v>
       </c>
       <c r="M42">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="43" spans="1:13">
       <c r="A43" s="1">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
@@ -2295,36 +2298,36 @@
         <v>56</v>
       </c>
       <c r="D43">
-        <v>960</v>
+        <v>0.6</v>
       </c>
       <c r="E43">
-        <v>-300</v>
+        <v>0.15</v>
       </c>
       <c r="F43">
-        <v>425</v>
+        <v>-0.775</v>
       </c>
       <c r="G43">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H43">
         <v>1</v>
       </c>
       <c r="I43" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J43">
         <v>1</v>
       </c>
       <c r="L43">
-        <v>592</v>
+        <v>1.94</v>
       </c>
       <c r="M43">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="44" spans="1:13">
       <c r="A44" s="1">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B44" t="s">
         <v>14</v>
@@ -2333,13 +2336,13 @@
         <v>57</v>
       </c>
       <c r="D44">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="E44">
-        <v>750</v>
+        <v>-0.45</v>
       </c>
       <c r="F44">
-        <v>-25</v>
+        <v>-0.775</v>
       </c>
       <c r="G44">
         <v>5</v>
@@ -2348,16 +2351,16 @@
         <v>1</v>
       </c>
       <c r="I44" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J44">
         <v>1</v>
       </c>
       <c r="L44">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M44">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -2371,13 +2374,13 @@
         <v>58</v>
       </c>
       <c r="D45">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="E45">
-        <v>150</v>
+        <v>0.15</v>
       </c>
       <c r="F45">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G45">
         <v>5</v>
@@ -2386,21 +2389,21 @@
         <v>1</v>
       </c>
       <c r="I45" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J45">
         <v>1</v>
       </c>
       <c r="L45">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M45">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="46" spans="1:13">
       <c r="A46" s="1">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
@@ -2409,13 +2412,13 @@
         <v>59</v>
       </c>
       <c r="D46">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="E46">
-        <v>150</v>
+        <v>0.75</v>
       </c>
       <c r="F46">
-        <v>-775</v>
+        <v>-0.025</v>
       </c>
       <c r="G46">
         <v>5</v>
@@ -2424,21 +2427,21 @@
         <v>1</v>
       </c>
       <c r="I46" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J46">
         <v>1</v>
       </c>
       <c r="L46">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M46">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="47" spans="1:13">
       <c r="A47" s="1">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B47" t="s">
         <v>14</v>
@@ -2447,13 +2450,13 @@
         <v>60</v>
       </c>
       <c r="D47">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="E47">
-        <v>-450</v>
+        <v>0.75</v>
       </c>
       <c r="F47">
-        <v>-25</v>
+        <v>-0.775</v>
       </c>
       <c r="G47">
         <v>5</v>
@@ -2462,21 +2465,21 @@
         <v>1</v>
       </c>
       <c r="I47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J47">
         <v>1</v>
       </c>
       <c r="L47">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M47">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="48" spans="1:13">
       <c r="A48" s="1">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B48" t="s">
         <v>14</v>
@@ -2485,13 +2488,13 @@
         <v>61</v>
       </c>
       <c r="D48">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="E48">
-        <v>-450</v>
+        <v>-0.9</v>
       </c>
       <c r="F48">
-        <v>-775</v>
+        <v>-0.025</v>
       </c>
       <c r="G48">
         <v>5</v>
@@ -2500,21 +2503,21 @@
         <v>1</v>
       </c>
       <c r="I48" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J48">
         <v>1</v>
       </c>
       <c r="L48">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M48">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="49" spans="1:13">
       <c r="A49" s="1">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -2523,13 +2526,13 @@
         <v>62</v>
       </c>
       <c r="D49">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="E49">
-        <v>-900</v>
+        <v>-0.9</v>
       </c>
       <c r="F49">
-        <v>-25</v>
+        <v>-0.775</v>
       </c>
       <c r="G49">
         <v>5</v>
@@ -2538,21 +2541,21 @@
         <v>1</v>
       </c>
       <c r="I49" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J49">
         <v>1</v>
       </c>
       <c r="L49">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M49">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="50" spans="1:13">
       <c r="A50" s="1">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B50" t="s">
         <v>14</v>
@@ -2561,13 +2564,13 @@
         <v>63</v>
       </c>
       <c r="D50">
-        <v>600</v>
+        <v>0.3</v>
       </c>
       <c r="E50">
-        <v>-900</v>
+        <v>-0.9</v>
       </c>
       <c r="F50">
-        <v>-775</v>
+        <v>0.425</v>
       </c>
       <c r="G50">
         <v>5</v>
@@ -2576,21 +2579,21 @@
         <v>1</v>
       </c>
       <c r="I50" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J50">
         <v>1</v>
       </c>
       <c r="L50">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M50">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="51" spans="1:13">
       <c r="A51" s="1">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="B51" t="s">
         <v>14</v>
@@ -2599,13 +2602,13 @@
         <v>64</v>
       </c>
       <c r="D51">
-        <v>600</v>
+        <v>0.3</v>
       </c>
       <c r="E51">
-        <v>750</v>
+        <v>-0.9</v>
       </c>
       <c r="F51">
-        <v>-775</v>
+        <v>-0.175</v>
       </c>
       <c r="G51">
         <v>5</v>
@@ -2614,21 +2617,21 @@
         <v>1</v>
       </c>
       <c r="I51" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J51">
         <v>1</v>
       </c>
       <c r="L51">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M51">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="52" spans="1:13">
       <c r="A52" s="1">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B52" t="s">
         <v>14</v>
@@ -2637,13 +2640,13 @@
         <v>65</v>
       </c>
       <c r="D52">
-        <v>300</v>
+        <v>0.3</v>
       </c>
       <c r="E52">
-        <v>-900</v>
+        <v>-0.9</v>
       </c>
       <c r="F52">
-        <v>425</v>
+        <v>-0.775</v>
       </c>
       <c r="G52">
         <v>5</v>
@@ -2652,16 +2655,16 @@
         <v>1</v>
       </c>
       <c r="I52" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J52">
         <v>1</v>
       </c>
       <c r="L52">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M52">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -2675,13 +2678,13 @@
         <v>66</v>
       </c>
       <c r="D53">
-        <v>300</v>
+        <v>0.3</v>
       </c>
       <c r="E53">
-        <v>-900</v>
+        <v>-0.9</v>
       </c>
       <c r="F53">
-        <v>1025</v>
+        <v>1.025</v>
       </c>
       <c r="G53">
         <v>5</v>
@@ -2690,21 +2693,21 @@
         <v>1</v>
       </c>
       <c r="I53" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J53">
         <v>1</v>
       </c>
       <c r="L53">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M53">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="54" spans="1:13">
       <c r="A54" s="1">
-        <v>201</v>
+        <v>224</v>
       </c>
       <c r="B54" t="s">
         <v>14</v>
@@ -2713,36 +2716,36 @@
         <v>67</v>
       </c>
       <c r="D54">
-        <v>300</v>
+        <v>1.8</v>
       </c>
       <c r="E54">
-        <v>-900</v>
+        <v>0.3</v>
       </c>
       <c r="F54">
-        <v>-775</v>
+        <v>1.05</v>
       </c>
       <c r="G54">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H54">
         <v>1</v>
       </c>
       <c r="I54" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J54">
         <v>1</v>
       </c>
       <c r="L54">
-        <v>1940</v>
+        <v>1.932</v>
       </c>
       <c r="M54">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="55" spans="1:13">
       <c r="A55" s="1">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="B55" t="s">
         <v>14</v>
@@ -2751,36 +2754,36 @@
         <v>68</v>
       </c>
       <c r="D55">
-        <v>300</v>
+        <v>1.8</v>
       </c>
       <c r="E55">
-        <v>-900</v>
+        <v>0.3</v>
       </c>
       <c r="F55">
-        <v>-175</v>
+        <v>0.45</v>
       </c>
       <c r="G55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H55">
         <v>1</v>
       </c>
       <c r="I55" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J55">
         <v>1</v>
       </c>
       <c r="L55">
-        <v>1940</v>
+        <v>1.932</v>
       </c>
       <c r="M55">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="56" spans="1:13">
       <c r="A56" s="1">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B56" t="s">
         <v>14</v>
@@ -2789,13 +2792,13 @@
         <v>69</v>
       </c>
       <c r="D56">
-        <v>1800</v>
+        <v>1.8</v>
       </c>
       <c r="E56">
-        <v>300</v>
+        <v>0.3</v>
       </c>
       <c r="F56">
-        <v>1050</v>
+        <v>-0.75</v>
       </c>
       <c r="G56">
         <v>6</v>
@@ -2804,16 +2807,16 @@
         <v>1</v>
       </c>
       <c r="I56" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J56">
         <v>1</v>
       </c>
       <c r="L56">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
       <c r="M56">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -2827,13 +2830,13 @@
         <v>70</v>
       </c>
       <c r="D57">
-        <v>1800</v>
+        <v>1.8</v>
       </c>
       <c r="E57">
-        <v>300</v>
+        <v>0.3</v>
       </c>
       <c r="F57">
-        <v>-150</v>
+        <v>-0.15</v>
       </c>
       <c r="G57">
         <v>6</v>
@@ -2842,21 +2845,21 @@
         <v>1</v>
       </c>
       <c r="I57" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J57">
         <v>1</v>
       </c>
       <c r="L57">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
       <c r="M57">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="58" spans="1:13">
       <c r="A58" s="1">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B58" t="s">
         <v>14</v>
@@ -2865,13 +2868,13 @@
         <v>71</v>
       </c>
       <c r="D58">
-        <v>1800</v>
+        <v>1.8</v>
       </c>
       <c r="E58">
-        <v>300</v>
+        <v>-0.3</v>
       </c>
       <c r="F58">
-        <v>450</v>
+        <v>0.45</v>
       </c>
       <c r="G58">
         <v>6</v>
@@ -2880,21 +2883,21 @@
         <v>1</v>
       </c>
       <c r="I58" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J58">
         <v>1</v>
       </c>
       <c r="L58">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
       <c r="M58">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="59" spans="1:13">
       <c r="A59" s="1">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B59" t="s">
         <v>14</v>
@@ -2903,13 +2906,13 @@
         <v>72</v>
       </c>
       <c r="D59">
-        <v>1800</v>
+        <v>1.8</v>
       </c>
       <c r="E59">
-        <v>-300</v>
+        <v>-0.3</v>
       </c>
       <c r="F59">
-        <v>1050</v>
+        <v>-0.15</v>
       </c>
       <c r="G59">
         <v>6</v>
@@ -2918,21 +2921,21 @@
         <v>1</v>
       </c>
       <c r="I59" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J59">
         <v>1</v>
       </c>
       <c r="L59">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
       <c r="M59">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="60" spans="1:13">
       <c r="A60" s="1">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B60" t="s">
         <v>14</v>
@@ -2941,13 +2944,13 @@
         <v>73</v>
       </c>
       <c r="D60">
-        <v>1800</v>
+        <v>1.8</v>
       </c>
       <c r="E60">
-        <v>-300</v>
+        <v>-0.3</v>
       </c>
       <c r="F60">
-        <v>450</v>
+        <v>-0.75</v>
       </c>
       <c r="G60">
         <v>6</v>
@@ -2956,21 +2959,21 @@
         <v>1</v>
       </c>
       <c r="I60" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J60">
         <v>1</v>
       </c>
       <c r="L60">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
       <c r="M60">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="61" spans="1:13">
       <c r="A61" s="1">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B61" t="s">
         <v>14</v>
@@ -2979,13 +2982,13 @@
         <v>74</v>
       </c>
       <c r="D61">
-        <v>1800</v>
+        <v>1.8</v>
       </c>
       <c r="E61">
-        <v>-300</v>
+        <v>-0.3</v>
       </c>
       <c r="F61">
-        <v>-150</v>
+        <v>1.05</v>
       </c>
       <c r="G61">
         <v>6</v>
@@ -2994,21 +2997,21 @@
         <v>1</v>
       </c>
       <c r="I61" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J61">
         <v>1</v>
       </c>
       <c r="L61">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
       <c r="M61">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="62" spans="1:13">
       <c r="A62" s="1">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="B62" t="s">
         <v>14</v>
@@ -3017,36 +3020,36 @@
         <v>75</v>
       </c>
       <c r="D62">
-        <v>1800</v>
+        <v>0.72</v>
       </c>
       <c r="E62">
-        <v>-300</v>
+        <v>0.6</v>
       </c>
       <c r="F62">
-        <v>-750</v>
-      </c>
-      <c r="G62">
-        <v>6</v>
+        <v>-0.025</v>
+      </c>
+      <c r="G62" t="s">
+        <v>87</v>
       </c>
       <c r="H62">
         <v>1</v>
       </c>
       <c r="I62" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J62">
         <v>1</v>
       </c>
       <c r="L62">
-        <v>1932</v>
+        <v>2.9</v>
       </c>
       <c r="M62">
-        <v>2655</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="63" spans="1:13">
       <c r="A63" s="1">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B63" t="s">
         <v>14</v>
@@ -3055,36 +3058,36 @@
         <v>76</v>
       </c>
       <c r="D63">
-        <v>1800</v>
+        <v>1.41</v>
       </c>
       <c r="E63">
-        <v>300</v>
+        <v>0.15</v>
       </c>
       <c r="F63">
-        <v>-750</v>
-      </c>
-      <c r="G63">
-        <v>6</v>
+        <v>-0.025</v>
+      </c>
+      <c r="G63" t="s">
+        <v>87</v>
       </c>
       <c r="H63">
         <v>1</v>
       </c>
       <c r="I63" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J63">
         <v>1</v>
       </c>
       <c r="L63">
-        <v>1932</v>
+        <v>2.9</v>
       </c>
       <c r="M63">
-        <v>2655</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="64" spans="1:13">
       <c r="A64" s="1">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="B64" t="s">
         <v>14</v>
@@ -3093,36 +3096,36 @@
         <v>77</v>
       </c>
       <c r="D64">
-        <v>720</v>
+        <v>1.41</v>
       </c>
       <c r="E64">
-        <v>1050</v>
+        <v>0.6</v>
       </c>
       <c r="F64">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G64" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H64">
         <v>1</v>
       </c>
       <c r="I64" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J64">
         <v>1</v>
       </c>
       <c r="L64">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M64">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="65" spans="1:13">
       <c r="A65" s="1">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="B65" t="s">
         <v>14</v>
@@ -3131,36 +3134,36 @@
         <v>78</v>
       </c>
       <c r="D65">
-        <v>720</v>
+        <v>1.41</v>
       </c>
       <c r="E65">
-        <v>600</v>
+        <v>1.2</v>
       </c>
       <c r="F65">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G65" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H65">
         <v>1</v>
       </c>
       <c r="I65" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J65">
         <v>1</v>
       </c>
       <c r="L65">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M65">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="66" spans="1:13">
       <c r="A66" s="1">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B66" t="s">
         <v>14</v>
@@ -3169,36 +3172,36 @@
         <v>79</v>
       </c>
       <c r="D66">
-        <v>720</v>
+        <v>2.31</v>
       </c>
       <c r="E66">
-        <v>150</v>
+        <v>0.15</v>
       </c>
       <c r="F66">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G66" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H66">
         <v>1</v>
       </c>
       <c r="I66" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J66">
         <v>1</v>
       </c>
       <c r="L66">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M66">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="67" spans="1:13">
       <c r="A67" s="1">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B67" t="s">
         <v>14</v>
@@ -3207,36 +3210,36 @@
         <v>80</v>
       </c>
       <c r="D67">
-        <v>120</v>
+        <v>2.31</v>
       </c>
       <c r="E67">
-        <v>150</v>
+        <v>0.6</v>
       </c>
       <c r="F67">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G67" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H67">
         <v>1</v>
       </c>
       <c r="I67" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J67">
         <v>1</v>
       </c>
       <c r="L67">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M67">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="68" spans="1:13">
       <c r="A68" s="1">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B68" t="s">
         <v>14</v>
@@ -3245,36 +3248,36 @@
         <v>81</v>
       </c>
       <c r="D68">
-        <v>120</v>
+        <v>2.31</v>
       </c>
       <c r="E68">
-        <v>600</v>
+        <v>1.2</v>
       </c>
       <c r="F68">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G68" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H68">
         <v>1</v>
       </c>
       <c r="I68" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J68">
         <v>1</v>
       </c>
       <c r="L68">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M68">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="69" spans="1:13">
       <c r="A69" s="1">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B69" t="s">
         <v>14</v>
@@ -3283,36 +3286,36 @@
         <v>82</v>
       </c>
       <c r="D69">
-        <v>2310</v>
+        <v>0.12</v>
       </c>
       <c r="E69">
-        <v>1200</v>
+        <v>1.05</v>
       </c>
       <c r="F69">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G69" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H69">
         <v>1</v>
       </c>
       <c r="I69" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J69">
         <v>1</v>
       </c>
       <c r="L69">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M69">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="70" spans="1:13">
       <c r="A70" s="1">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B70" t="s">
         <v>14</v>
@@ -3321,36 +3324,36 @@
         <v>83</v>
       </c>
       <c r="D70">
-        <v>2310</v>
+        <v>0.12</v>
       </c>
       <c r="E70">
-        <v>600</v>
+        <v>0.6</v>
       </c>
       <c r="F70">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G70" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H70">
         <v>1</v>
       </c>
       <c r="I70" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J70">
         <v>1</v>
       </c>
       <c r="L70">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M70">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="71" spans="1:13">
       <c r="A71" s="1">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B71" t="s">
         <v>14</v>
@@ -3359,36 +3362,36 @@
         <v>84</v>
       </c>
       <c r="D71">
-        <v>2310</v>
+        <v>0.12</v>
       </c>
       <c r="E71">
-        <v>150</v>
+        <v>0.15</v>
       </c>
       <c r="F71">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G71" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H71">
         <v>1</v>
       </c>
       <c r="I71" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J71">
         <v>1</v>
       </c>
       <c r="L71">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M71">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="72" spans="1:13">
       <c r="A72" s="1">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B72" t="s">
         <v>14</v>
@@ -3397,36 +3400,36 @@
         <v>85</v>
       </c>
       <c r="D72">
-        <v>1410</v>
+        <v>0.72</v>
       </c>
       <c r="E72">
-        <v>1200</v>
+        <v>0.15</v>
       </c>
       <c r="F72">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G72" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H72">
         <v>1</v>
       </c>
       <c r="I72" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J72">
         <v>1</v>
       </c>
       <c r="L72">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M72">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
     <row r="73" spans="1:13">
       <c r="A73" s="1">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="B73" t="s">
         <v>14</v>
@@ -3435,107 +3438,31 @@
         <v>86</v>
       </c>
       <c r="D73">
-        <v>1410</v>
+        <v>0.72</v>
       </c>
       <c r="E73">
-        <v>150</v>
+        <v>1.05</v>
       </c>
       <c r="F73">
-        <v>-25</v>
+        <v>-0.025</v>
       </c>
       <c r="G73" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H73">
         <v>1</v>
       </c>
       <c r="I73" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J73">
         <v>1</v>
       </c>
       <c r="L73">
-        <v>2900</v>
+        <v>2.9</v>
       </c>
       <c r="M73">
-        <v>1932</v>
-      </c>
-    </row>
-    <row r="74" spans="1:13">
-      <c r="A74" s="1">
-        <v>231</v>
-      </c>
-      <c r="B74" t="s">
-        <v>14</v>
-      </c>
-      <c r="C74" t="s">
-        <v>87</v>
-      </c>
-      <c r="D74">
-        <v>120</v>
-      </c>
-      <c r="E74">
-        <v>1050</v>
-      </c>
-      <c r="F74">
-        <v>-25</v>
-      </c>
-      <c r="G74" t="s">
-        <v>89</v>
-      </c>
-      <c r="H74">
-        <v>1</v>
-      </c>
-      <c r="I74" t="s">
-        <v>91</v>
-      </c>
-      <c r="J74">
-        <v>1</v>
-      </c>
-      <c r="L74">
-        <v>2900</v>
-      </c>
-      <c r="M74">
-        <v>1932</v>
-      </c>
-    </row>
-    <row r="75" spans="1:13">
-      <c r="A75" s="1">
-        <v>226</v>
-      </c>
-      <c r="B75" t="s">
-        <v>14</v>
-      </c>
-      <c r="C75" t="s">
-        <v>88</v>
-      </c>
-      <c r="D75">
-        <v>1410</v>
-      </c>
-      <c r="E75">
-        <v>600</v>
-      </c>
-      <c r="F75">
-        <v>-25</v>
-      </c>
-      <c r="G75" t="s">
-        <v>89</v>
-      </c>
-      <c r="H75">
-        <v>1</v>
-      </c>
-      <c r="I75" t="s">
-        <v>91</v>
-      </c>
-      <c r="J75">
-        <v>1</v>
-      </c>
-      <c r="L75">
-        <v>2900</v>
-      </c>
-      <c r="M75">
-        <v>1932</v>
+        <v>1.932</v>
       </c>
     </row>
   </sheetData>
@@ -3597,19 +3524,19 @@
         <v>164</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D2">
-        <v>1202</v>
+        <v>1.202</v>
       </c>
       <c r="E2">
-        <v>160</v>
+        <v>0.16</v>
       </c>
       <c r="F2">
-        <v>-181</v>
+        <v>-0.181</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -3618,16 +3545,16 @@
         <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="L2">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M2">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -3635,19 +3562,19 @@
         <v>146</v>
       </c>
       <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
         <v>92</v>
       </c>
-      <c r="C3" t="s">
-        <v>94</v>
-      </c>
       <c r="D3">
-        <v>1200</v>
+        <v>1.2</v>
       </c>
       <c r="E3">
-        <v>210</v>
+        <v>0.21</v>
       </c>
       <c r="F3">
-        <v>-50</v>
+        <v>-0.05</v>
       </c>
       <c r="G3">
         <v>3</v>
@@ -3656,36 +3583,36 @@
         <v>6</v>
       </c>
       <c r="I3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>960</v>
+        <v>0.96</v>
       </c>
       <c r="M3">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1">
-        <v>158</v>
+        <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D4">
-        <v>392</v>
+        <v>0.305</v>
       </c>
       <c r="E4">
-        <v>-575</v>
+        <v>0.45</v>
       </c>
       <c r="F4">
-        <v>-1024</v>
+        <v>-0.453</v>
       </c>
       <c r="G4">
         <v>5</v>
@@ -3694,36 +3621,36 @@
         <v>6</v>
       </c>
       <c r="I4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M4">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="1">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D5">
-        <v>492</v>
+        <v>0.392</v>
       </c>
       <c r="E5">
-        <v>-450</v>
+        <v>-0.575</v>
       </c>
       <c r="F5">
-        <v>-175</v>
+        <v>-1.024</v>
       </c>
       <c r="G5">
         <v>5</v>
@@ -3732,36 +3659,36 @@
         <v>6</v>
       </c>
       <c r="I5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J5">
         <v>1</v>
       </c>
       <c r="L5">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M5">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="1">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D6">
-        <v>540</v>
+        <v>0.492</v>
       </c>
       <c r="E6">
-        <v>450</v>
+        <v>-0.45</v>
       </c>
       <c r="F6">
-        <v>-175</v>
+        <v>-0.175</v>
       </c>
       <c r="G6">
         <v>5</v>
@@ -3770,36 +3697,36 @@
         <v>6</v>
       </c>
       <c r="I6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J6">
         <v>1</v>
       </c>
       <c r="L6">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M6">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="1">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D7">
-        <v>305</v>
+        <v>0.54</v>
       </c>
       <c r="E7">
-        <v>450</v>
+        <v>0.45</v>
       </c>
       <c r="F7">
-        <v>-453</v>
+        <v>-0.175</v>
       </c>
       <c r="G7">
         <v>5</v>
@@ -3808,36 +3735,36 @@
         <v>6</v>
       </c>
       <c r="I7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="L7">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M7">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="1">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D8">
-        <v>600</v>
+        <v>0.38</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="F8">
-        <v>125</v>
+        <v>-0.725</v>
       </c>
       <c r="G8">
         <v>5</v>
@@ -3846,36 +3773,36 @@
         <v>6</v>
       </c>
       <c r="I8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J8">
         <v>1</v>
       </c>
       <c r="L8">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M8">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="1">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D9">
-        <v>380</v>
+        <v>0.6</v>
       </c>
       <c r="E9">
-        <v>-800</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>-725</v>
+        <v>0.125</v>
       </c>
       <c r="G9">
         <v>5</v>
@@ -3884,16 +3811,16 @@
         <v>6</v>
       </c>
       <c r="I9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J9">
         <v>1</v>
       </c>
       <c r="L9">
-        <v>1940</v>
+        <v>1.94</v>
       </c>
       <c r="M9">
-        <v>2655</v>
+        <v>2.655</v>
       </c>
     </row>
   </sheetData>
@@ -3914,13 +3841,13 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>101</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>

</xml_diff>